<commit_message>
Improve inventory adjustment form and preserve binary assets
</commit_message>
<xml_diff>
--- a/downloads/inventory/dixani-inventory-adjustment-form.xlsx
+++ b/downloads/inventory/dixani-inventory-adjustment-form.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustment Form" sheetId="1" r:id="R5d4ccb136d0f47ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="R4a30822c6ca84f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R814a8c76d95b48fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adjustment Form" sheetId="1" r:id="R48f077245b22421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" r:id="Re58070100e614840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R83b04f1ce7814959"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,7 +240,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -251,7 +251,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -555,13 +555,13 @@
         <x:v>Currency</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>QAR</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="L5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>Adjustment Type</x:v>
+        <x:v>Type</x:v>
       </x:c>
       <x:c r="B6" t="str">
         <x:v>Stock Variance</x:v>
@@ -625,14 +625,14 @@
       <x:c r="C10" s="26" t="str"/>
       <x:c r="D10" s="26" t="str"/>
       <x:c r="E10" s="26" t="str"/>
-      <x:c r="F10" s="46" t="str"/>
-      <x:c r="G10" s="46" t="str"/>
+      <x:c r="F10" s="46"/>
+      <x:c r="G10" s="46"/>
       <x:c r="H10" s="46" t="str">
-        <x:f>IF(OR(F10="",G10=""),"",G10-F10)</x:f>
-      </x:c>
-      <x:c r="I10" s="50" t="str"/>
+        <x:f>IF(AND(ISNUMBER(F10),ISNUMBER(G10)),G10-F10,"")</x:f>
+      </x:c>
+      <x:c r="I10" s="50"/>
       <x:c r="J10" s="50" t="str">
-        <x:f>IF(OR(H10="",I10=""),"",H10*I10)</x:f>
+        <x:f>IF(AND(ISNUMBER(H10),ISNUMBER(I10)),H10*I10,"")</x:f>
       </x:c>
       <x:c r="K10" s="26" t="str"/>
       <x:c r="L10" s="26" t="str"/>
@@ -648,11 +648,11 @@
       <x:c r="F11" s="47" t="str"/>
       <x:c r="G11" s="47" t="str"/>
       <x:c r="H11" s="47" t="str">
-        <x:f>IF(OR(F11="",G11=""),"",G11-F11)</x:f>
+        <x:f>IF(AND(ISNUMBER(F11),ISNUMBER(G11)),G11-F11,"")</x:f>
       </x:c>
       <x:c r="I11" s="51" t="str"/>
       <x:c r="J11" s="51" t="str">
-        <x:f>IF(OR(H11="",I11=""),"",H11*I11)</x:f>
+        <x:f>IF(AND(ISNUMBER(H11),ISNUMBER(I11)),H11*I11,"")</x:f>
       </x:c>
       <x:c r="K11" s="28" t="str"/>
       <x:c r="L11" s="28" t="str"/>
@@ -668,11 +668,11 @@
       <x:c r="F12" s="46" t="str"/>
       <x:c r="G12" s="46" t="str"/>
       <x:c r="H12" s="46" t="str">
-        <x:f>IF(OR(F12="",G12=""),"",G12-F12)</x:f>
+        <x:f>IF(AND(ISNUMBER(F12),ISNUMBER(G12)),G12-F12,"")</x:f>
       </x:c>
       <x:c r="I12" s="50" t="str"/>
       <x:c r="J12" s="50" t="str">
-        <x:f>IF(OR(H12="",I12=""),"",H12*I12)</x:f>
+        <x:f>IF(AND(ISNUMBER(H12),ISNUMBER(I12)),H12*I12,"")</x:f>
       </x:c>
       <x:c r="K12" s="26" t="str"/>
       <x:c r="L12" s="26" t="str"/>
@@ -688,11 +688,11 @@
       <x:c r="F13" s="47" t="str"/>
       <x:c r="G13" s="47" t="str"/>
       <x:c r="H13" s="47" t="str">
-        <x:f>IF(OR(F13="",G13=""),"",G13-F13)</x:f>
+        <x:f>IF(AND(ISNUMBER(F13),ISNUMBER(G13)),G13-F13,"")</x:f>
       </x:c>
       <x:c r="I13" s="51" t="str"/>
       <x:c r="J13" s="51" t="str">
-        <x:f>IF(OR(H13="",I13=""),"",H13*I13)</x:f>
+        <x:f>IF(AND(ISNUMBER(H13),ISNUMBER(I13)),H13*I13,"")</x:f>
       </x:c>
       <x:c r="K13" s="28" t="str"/>
       <x:c r="L13" s="28" t="str"/>
@@ -708,11 +708,11 @@
       <x:c r="F14" s="46" t="str"/>
       <x:c r="G14" s="46" t="str"/>
       <x:c r="H14" s="46" t="str">
-        <x:f>IF(OR(F14="",G14=""),"",G14-F14)</x:f>
+        <x:f>IF(AND(ISNUMBER(F14),ISNUMBER(G14)),G14-F14,"")</x:f>
       </x:c>
       <x:c r="I14" s="50" t="str"/>
       <x:c r="J14" s="50" t="str">
-        <x:f>IF(OR(H14="",I14=""),"",H14*I14)</x:f>
+        <x:f>IF(AND(ISNUMBER(H14),ISNUMBER(I14)),H14*I14,"")</x:f>
       </x:c>
       <x:c r="K14" s="26" t="str"/>
       <x:c r="L14" s="26" t="str"/>
@@ -728,11 +728,11 @@
       <x:c r="F15" s="47" t="str"/>
       <x:c r="G15" s="47" t="str"/>
       <x:c r="H15" s="47" t="str">
-        <x:f>IF(OR(F15="",G15=""),"",G15-F15)</x:f>
+        <x:f>IF(AND(ISNUMBER(F15),ISNUMBER(G15)),G15-F15,"")</x:f>
       </x:c>
       <x:c r="I15" s="51" t="str"/>
       <x:c r="J15" s="51" t="str">
-        <x:f>IF(OR(H15="",I15=""),"",H15*I15)</x:f>
+        <x:f>IF(AND(ISNUMBER(H15),ISNUMBER(I15)),H15*I15,"")</x:f>
       </x:c>
       <x:c r="K15" s="28" t="str"/>
       <x:c r="L15" s="28" t="str"/>
@@ -748,11 +748,11 @@
       <x:c r="F16" s="46" t="str"/>
       <x:c r="G16" s="46" t="str"/>
       <x:c r="H16" s="46" t="str">
-        <x:f>IF(OR(F16="",G16=""),"",G16-F16)</x:f>
+        <x:f>IF(AND(ISNUMBER(F16),ISNUMBER(G16)),G16-F16,"")</x:f>
       </x:c>
       <x:c r="I16" s="50" t="str"/>
       <x:c r="J16" s="50" t="str">
-        <x:f>IF(OR(H16="",I16=""),"",H16*I16)</x:f>
+        <x:f>IF(AND(ISNUMBER(H16),ISNUMBER(I16)),H16*I16,"")</x:f>
       </x:c>
       <x:c r="K16" s="26" t="str"/>
       <x:c r="L16" s="26" t="str"/>
@@ -768,11 +768,11 @@
       <x:c r="F17" s="47" t="str"/>
       <x:c r="G17" s="47" t="str"/>
       <x:c r="H17" s="47" t="str">
-        <x:f>IF(OR(F17="",G17=""),"",G17-F17)</x:f>
+        <x:f>IF(AND(ISNUMBER(F17),ISNUMBER(G17)),G17-F17,"")</x:f>
       </x:c>
       <x:c r="I17" s="51" t="str"/>
       <x:c r="J17" s="51" t="str">
-        <x:f>IF(OR(H17="",I17=""),"",H17*I17)</x:f>
+        <x:f>IF(AND(ISNUMBER(H17),ISNUMBER(I17)),H17*I17,"")</x:f>
       </x:c>
       <x:c r="K17" s="28" t="str"/>
       <x:c r="L17" s="28" t="str"/>
@@ -788,11 +788,11 @@
       <x:c r="F18" s="46" t="str"/>
       <x:c r="G18" s="46" t="str"/>
       <x:c r="H18" s="46" t="str">
-        <x:f>IF(OR(F18="",G18=""),"",G18-F18)</x:f>
+        <x:f>IF(AND(ISNUMBER(F18),ISNUMBER(G18)),G18-F18,"")</x:f>
       </x:c>
       <x:c r="I18" s="50" t="str"/>
       <x:c r="J18" s="50" t="str">
-        <x:f>IF(OR(H18="",I18=""),"",H18*I18)</x:f>
+        <x:f>IF(AND(ISNUMBER(H18),ISNUMBER(I18)),H18*I18,"")</x:f>
       </x:c>
       <x:c r="K18" s="26" t="str"/>
       <x:c r="L18" s="26" t="str"/>
@@ -808,11 +808,11 @@
       <x:c r="F19" s="47" t="str"/>
       <x:c r="G19" s="47" t="str"/>
       <x:c r="H19" s="47" t="str">
-        <x:f>IF(OR(F19="",G19=""),"",G19-F19)</x:f>
+        <x:f>IF(AND(ISNUMBER(F19),ISNUMBER(G19)),G19-F19,"")</x:f>
       </x:c>
       <x:c r="I19" s="51" t="str"/>
       <x:c r="J19" s="51" t="str">
-        <x:f>IF(OR(H19="",I19=""),"",H19*I19)</x:f>
+        <x:f>IF(AND(ISNUMBER(H19),ISNUMBER(I19)),H19*I19,"")</x:f>
       </x:c>
       <x:c r="K19" s="28" t="str"/>
       <x:c r="L19" s="28" t="str"/>
@@ -828,11 +828,11 @@
       <x:c r="F20" s="46" t="str"/>
       <x:c r="G20" s="46" t="str"/>
       <x:c r="H20" s="46" t="str">
-        <x:f>IF(OR(F20="",G20=""),"",G20-F20)</x:f>
+        <x:f>IF(AND(ISNUMBER(F20),ISNUMBER(G20)),G20-F20,"")</x:f>
       </x:c>
       <x:c r="I20" s="50" t="str"/>
       <x:c r="J20" s="50" t="str">
-        <x:f>IF(OR(H20="",I20=""),"",H20*I20)</x:f>
+        <x:f>IF(AND(ISNUMBER(H20),ISNUMBER(I20)),H20*I20,"")</x:f>
       </x:c>
       <x:c r="K20" s="26" t="str"/>
       <x:c r="L20" s="26" t="str"/>
@@ -848,11 +848,11 @@
       <x:c r="F21" s="47" t="str"/>
       <x:c r="G21" s="47" t="str"/>
       <x:c r="H21" s="47" t="str">
-        <x:f>IF(OR(F21="",G21=""),"",G21-F21)</x:f>
+        <x:f>IF(AND(ISNUMBER(F21),ISNUMBER(G21)),G21-F21,"")</x:f>
       </x:c>
       <x:c r="I21" s="51" t="str"/>
       <x:c r="J21" s="51" t="str">
-        <x:f>IF(OR(H21="",I21=""),"",H21*I21)</x:f>
+        <x:f>IF(AND(ISNUMBER(H21),ISNUMBER(I21)),H21*I21,"")</x:f>
       </x:c>
       <x:c r="K21" s="28" t="str"/>
       <x:c r="L21" s="28" t="str"/>
@@ -868,11 +868,11 @@
       <x:c r="F22" s="46" t="str"/>
       <x:c r="G22" s="46" t="str"/>
       <x:c r="H22" s="46" t="str">
-        <x:f>IF(OR(F22="",G22=""),"",G22-F22)</x:f>
+        <x:f>IF(AND(ISNUMBER(F22),ISNUMBER(G22)),G22-F22,"")</x:f>
       </x:c>
       <x:c r="I22" s="50" t="str"/>
       <x:c r="J22" s="50" t="str">
-        <x:f>IF(OR(H22="",I22=""),"",H22*I22)</x:f>
+        <x:f>IF(AND(ISNUMBER(H22),ISNUMBER(I22)),H22*I22,"")</x:f>
       </x:c>
       <x:c r="K22" s="26" t="str"/>
       <x:c r="L22" s="26" t="str"/>
@@ -888,11 +888,11 @@
       <x:c r="F23" s="47" t="str"/>
       <x:c r="G23" s="47" t="str"/>
       <x:c r="H23" s="47" t="str">
-        <x:f>IF(OR(F23="",G23=""),"",G23-F23)</x:f>
+        <x:f>IF(AND(ISNUMBER(F23),ISNUMBER(G23)),G23-F23,"")</x:f>
       </x:c>
       <x:c r="I23" s="51" t="str"/>
       <x:c r="J23" s="51" t="str">
-        <x:f>IF(OR(H23="",I23=""),"",H23*I23)</x:f>
+        <x:f>IF(AND(ISNUMBER(H23),ISNUMBER(I23)),H23*I23,"")</x:f>
       </x:c>
       <x:c r="K23" s="28" t="str"/>
       <x:c r="L23" s="28" t="str"/>
@@ -908,11 +908,11 @@
       <x:c r="F24" s="46" t="str"/>
       <x:c r="G24" s="46" t="str"/>
       <x:c r="H24" s="46" t="str">
-        <x:f>IF(OR(F24="",G24=""),"",G24-F24)</x:f>
+        <x:f>IF(AND(ISNUMBER(F24),ISNUMBER(G24)),G24-F24,"")</x:f>
       </x:c>
       <x:c r="I24" s="50" t="str"/>
       <x:c r="J24" s="50" t="str">
-        <x:f>IF(OR(H24="",I24=""),"",H24*I24)</x:f>
+        <x:f>IF(AND(ISNUMBER(H24),ISNUMBER(I24)),H24*I24,"")</x:f>
       </x:c>
       <x:c r="K24" s="26" t="str"/>
       <x:c r="L24" s="26" t="str"/>
@@ -928,11 +928,11 @@
       <x:c r="F25" s="47" t="str"/>
       <x:c r="G25" s="47" t="str"/>
       <x:c r="H25" s="47" t="str">
-        <x:f>IF(OR(F25="",G25=""),"",G25-F25)</x:f>
+        <x:f>IF(AND(ISNUMBER(F25),ISNUMBER(G25)),G25-F25,"")</x:f>
       </x:c>
       <x:c r="I25" s="51" t="str"/>
       <x:c r="J25" s="51" t="str">
-        <x:f>IF(OR(H25="",I25=""),"",H25*I25)</x:f>
+        <x:f>IF(AND(ISNUMBER(H25),ISNUMBER(I25)),H25*I25,"")</x:f>
       </x:c>
       <x:c r="K25" s="28" t="str"/>
       <x:c r="L25" s="28" t="str"/>
@@ -948,11 +948,11 @@
       <x:c r="F26" s="46" t="str"/>
       <x:c r="G26" s="46" t="str"/>
       <x:c r="H26" s="46" t="str">
-        <x:f>IF(OR(F26="",G26=""),"",G26-F26)</x:f>
+        <x:f>IF(AND(ISNUMBER(F26),ISNUMBER(G26)),G26-F26,"")</x:f>
       </x:c>
       <x:c r="I26" s="50" t="str"/>
       <x:c r="J26" s="50" t="str">
-        <x:f>IF(OR(H26="",I26=""),"",H26*I26)</x:f>
+        <x:f>IF(AND(ISNUMBER(H26),ISNUMBER(I26)),H26*I26,"")</x:f>
       </x:c>
       <x:c r="K26" s="26" t="str"/>
       <x:c r="L26" s="26" t="str"/>
@@ -968,11 +968,11 @@
       <x:c r="F27" s="47" t="str"/>
       <x:c r="G27" s="47" t="str"/>
       <x:c r="H27" s="47" t="str">
-        <x:f>IF(OR(F27="",G27=""),"",G27-F27)</x:f>
+        <x:f>IF(AND(ISNUMBER(F27),ISNUMBER(G27)),G27-F27,"")</x:f>
       </x:c>
       <x:c r="I27" s="51" t="str"/>
       <x:c r="J27" s="51" t="str">
-        <x:f>IF(OR(H27="",I27=""),"",H27*I27)</x:f>
+        <x:f>IF(AND(ISNUMBER(H27),ISNUMBER(I27)),H27*I27,"")</x:f>
       </x:c>
       <x:c r="K27" s="28" t="str"/>
       <x:c r="L27" s="28" t="str"/>
@@ -988,11 +988,11 @@
       <x:c r="F28" s="46" t="str"/>
       <x:c r="G28" s="46" t="str"/>
       <x:c r="H28" s="46" t="str">
-        <x:f>IF(OR(F28="",G28=""),"",G28-F28)</x:f>
+        <x:f>IF(AND(ISNUMBER(F28),ISNUMBER(G28)),G28-F28,"")</x:f>
       </x:c>
       <x:c r="I28" s="50" t="str"/>
       <x:c r="J28" s="50" t="str">
-        <x:f>IF(OR(H28="",I28=""),"",H28*I28)</x:f>
+        <x:f>IF(AND(ISNUMBER(H28),ISNUMBER(I28)),H28*I28,"")</x:f>
       </x:c>
       <x:c r="K28" s="26" t="str"/>
       <x:c r="L28" s="26" t="str"/>
@@ -1008,11 +1008,11 @@
       <x:c r="F29" s="47" t="str"/>
       <x:c r="G29" s="47" t="str"/>
       <x:c r="H29" s="47" t="str">
-        <x:f>IF(OR(F29="",G29=""),"",G29-F29)</x:f>
+        <x:f>IF(AND(ISNUMBER(F29),ISNUMBER(G29)),G29-F29,"")</x:f>
       </x:c>
       <x:c r="I29" s="51" t="str"/>
       <x:c r="J29" s="51" t="str">
-        <x:f>IF(OR(H29="",I29=""),"",H29*I29)</x:f>
+        <x:f>IF(AND(ISNUMBER(H29),ISNUMBER(I29)),H29*I29,"")</x:f>
       </x:c>
       <x:c r="K29" s="28" t="str"/>
       <x:c r="L29" s="28" t="str"/>
@@ -1028,11 +1028,11 @@
       <x:c r="F30" s="46" t="str"/>
       <x:c r="G30" s="46" t="str"/>
       <x:c r="H30" s="46" t="str">
-        <x:f>IF(OR(F30="",G30=""),"",G30-F30)</x:f>
+        <x:f>IF(AND(ISNUMBER(F30),ISNUMBER(G30)),G30-F30,"")</x:f>
       </x:c>
       <x:c r="I30" s="50" t="str"/>
       <x:c r="J30" s="50" t="str">
-        <x:f>IF(OR(H30="",I30=""),"",H30*I30)</x:f>
+        <x:f>IF(AND(ISNUMBER(H30),ISNUMBER(I30)),H30*I30,"")</x:f>
       </x:c>
       <x:c r="K30" s="26" t="str"/>
       <x:c r="L30" s="26" t="str"/>
@@ -1048,11 +1048,11 @@
       <x:c r="F31" s="47" t="str"/>
       <x:c r="G31" s="47" t="str"/>
       <x:c r="H31" s="47" t="str">
-        <x:f>IF(OR(F31="",G31=""),"",G31-F31)</x:f>
+        <x:f>IF(AND(ISNUMBER(F31),ISNUMBER(G31)),G31-F31,"")</x:f>
       </x:c>
       <x:c r="I31" s="51" t="str"/>
       <x:c r="J31" s="51" t="str">
-        <x:f>IF(OR(H31="",I31=""),"",H31*I31)</x:f>
+        <x:f>IF(AND(ISNUMBER(H31),ISNUMBER(I31)),H31*I31,"")</x:f>
       </x:c>
       <x:c r="K31" s="28" t="str"/>
       <x:c r="L31" s="28" t="str"/>
@@ -1068,11 +1068,11 @@
       <x:c r="F32" s="46" t="str"/>
       <x:c r="G32" s="46" t="str"/>
       <x:c r="H32" s="46" t="str">
-        <x:f>IF(OR(F32="",G32=""),"",G32-F32)</x:f>
+        <x:f>IF(AND(ISNUMBER(F32),ISNUMBER(G32)),G32-F32,"")</x:f>
       </x:c>
       <x:c r="I32" s="50" t="str"/>
       <x:c r="J32" s="50" t="str">
-        <x:f>IF(OR(H32="",I32=""),"",H32*I32)</x:f>
+        <x:f>IF(AND(ISNUMBER(H32),ISNUMBER(I32)),H32*I32,"")</x:f>
       </x:c>
       <x:c r="K32" s="26" t="str"/>
       <x:c r="L32" s="26" t="str"/>
@@ -1088,11 +1088,11 @@
       <x:c r="F33" s="47" t="str"/>
       <x:c r="G33" s="47" t="str"/>
       <x:c r="H33" s="47" t="str">
-        <x:f>IF(OR(F33="",G33=""),"",G33-F33)</x:f>
+        <x:f>IF(AND(ISNUMBER(F33),ISNUMBER(G33)),G33-F33,"")</x:f>
       </x:c>
       <x:c r="I33" s="51" t="str"/>
       <x:c r="J33" s="51" t="str">
-        <x:f>IF(OR(H33="",I33=""),"",H33*I33)</x:f>
+        <x:f>IF(AND(ISNUMBER(H33),ISNUMBER(I33)),H33*I33,"")</x:f>
       </x:c>
       <x:c r="K33" s="28" t="str"/>
       <x:c r="L33" s="28" t="str"/>
@@ -1105,14 +1105,14 @@
       <x:c r="C34" s="26" t="str"/>
       <x:c r="D34" s="26" t="str"/>
       <x:c r="E34" s="26" t="str"/>
-      <x:c r="F34" s="46" t="str"/>
-      <x:c r="G34" s="46" t="str"/>
+      <x:c r="F34" s="46"/>
+      <x:c r="G34" s="46"/>
       <x:c r="H34" s="46" t="str">
-        <x:f>IF(OR(F34="",G34=""),"",G34-F34)</x:f>
-      </x:c>
-      <x:c r="I34" s="50" t="str"/>
+        <x:f>IF(AND(ISNUMBER(F34),ISNUMBER(G34)),G34-F34,"")</x:f>
+      </x:c>
+      <x:c r="I34" s="50"/>
       <x:c r="J34" s="50" t="str">
-        <x:f>IF(OR(H34="",I34=""),"",H34*I34)</x:f>
+        <x:f>IF(AND(ISNUMBER(H34),ISNUMBER(I34)),H34*I34,"")</x:f>
       </x:c>
       <x:c r="K34" s="26" t="str"/>
       <x:c r="L34" s="26" t="str"/>
@@ -1135,7 +1135,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="35" t="str">
-        <x:v>Total Lines</x:v>
+        <x:v>Calculated Lines</x:v>
       </x:c>
       <x:c r="B38" s="35" t="str"/>
       <x:c r="C38" s="35" t="str">
@@ -1161,8 +1161,8 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="41" t="n">
-        <x:f>COUNTIF(H10:H34,"&lt;&gt;")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNT(H10:H34)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B39" s="41"/>
       <x:c r="C39" s="41" t="n">
@@ -1176,17 +1176,17 @@
       </x:c>
       <x:c r="F39" s="41"/>
       <x:c r="G39" s="54" t="n">
-        <x:f>SUMIF(J10:J34,"&gt;0",J10:J34)</x:f>
+        <x:f>IF(COUNT(H10:H34)&lt;&gt;COUNT(J10:J34),"Incomplete",SUMIF(J10:J34,"&gt;0",J10:J34))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H39" s="54"/>
       <x:c r="I39" s="54" t="n">
-        <x:f>-SUMIF(J10:J34,"&lt;0",J10:J34)</x:f>
+        <x:f>IF(COUNT(H10:H34)&lt;&gt;COUNT(J10:J34),"Incomplete",-SUMIF(J10:J34,"&lt;0",J10:J34))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J39" s="54"/>
       <x:c r="K39" s="54" t="n">
-        <x:f>SUM(J10:J34)</x:f>
+        <x:f>IF(COUNT(H10:H34)&lt;&gt;COUNT(J10:J34),"Incomplete",SUM(J10:J34))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L39" s="54"/>
@@ -1207,12 +1207,12 @@
       <x:c r="K42" s="30"/>
       <x:c r="L42" s="30"/>
     </x:row>
-    <x:row r="43">
+    <x:row r="43" ht="32" customHeight="1">
       <x:c r="A43" s="34" t="str">
         <x:v>Root Cause / Investigation Summary</x:v>
       </x:c>
-      <x:c r="B43" t="str"/>
-      <x:c r="C43" t="str"/>
+      <x:c r="B43" s="26" t="str"/>
+      <x:c r="C43" s="26" t="str"/>
       <x:c r="D43" t="str"/>
       <x:c r="E43" t="str"/>
       <x:c r="F43" t="str"/>
@@ -1223,12 +1223,12 @@
       <x:c r="K43" t="str"/>
       <x:c r="L43" t="str"/>
     </x:row>
-    <x:row r="44">
+    <x:row r="44" ht="32" customHeight="1">
       <x:c r="A44" s="34" t="str">
         <x:v>Corrective Action</x:v>
       </x:c>
-      <x:c r="B44" t="str"/>
-      <x:c r="C44" t="str"/>
+      <x:c r="B44" s="26" t="str"/>
+      <x:c r="C44" s="26" t="str"/>
       <x:c r="D44" t="str"/>
       <x:c r="E44" t="str"/>
       <x:c r="F44" t="str"/>
@@ -1239,12 +1239,12 @@
       <x:c r="K44" t="str"/>
       <x:c r="L44" t="str"/>
     </x:row>
-    <x:row r="45">
+    <x:row r="45" ht="32" customHeight="1">
       <x:c r="A45" s="34" t="str">
         <x:v>Preventive Action</x:v>
       </x:c>
-      <x:c r="B45" t="str"/>
-      <x:c r="C45" t="str"/>
+      <x:c r="B45" s="26" t="str"/>
+      <x:c r="C45" s="26" t="str"/>
       <x:c r="D45" t="str"/>
       <x:c r="E45" t="str"/>
       <x:c r="F45" t="str"/>
@@ -1255,12 +1255,12 @@
       <x:c r="K45" t="str"/>
       <x:c r="L45" t="str"/>
     </x:row>
-    <x:row r="46">
+    <x:row r="46" ht="32" customHeight="1">
       <x:c r="A46" s="34" t="str">
         <x:v>Supporting Reference / Evidence</x:v>
       </x:c>
-      <x:c r="B46" t="str"/>
-      <x:c r="C46" t="str"/>
+      <x:c r="B46" s="26" t="str"/>
+      <x:c r="C46" s="26" t="str"/>
       <x:c r="D46" t="str"/>
       <x:c r="E46" t="str"/>
       <x:c r="F46" t="str"/>
@@ -1271,12 +1271,12 @@
       <x:c r="K46" t="str"/>
       <x:c r="L46" t="str"/>
     </x:row>
-    <x:row r="47">
+    <x:row r="47" ht="32" customHeight="1">
       <x:c r="A47" s="34" t="str">
         <x:v>Approval Notes</x:v>
       </x:c>
-      <x:c r="B47" t="str"/>
-      <x:c r="C47" t="str"/>
+      <x:c r="B47" s="26" t="str"/>
+      <x:c r="C47" s="26" t="str"/>
       <x:c r="D47" t="str"/>
       <x:c r="E47" t="str"/>
       <x:c r="F47" t="str"/>
@@ -1335,17 +1335,22 @@
     <x:mergeCell ref="I39:J39"/>
     <x:mergeCell ref="K39:L39"/>
     <x:mergeCell ref="A42:L42"/>
-    <x:mergeCell ref="B43:L43"/>
-    <x:mergeCell ref="B44:L44"/>
-    <x:mergeCell ref="B45:L45"/>
-    <x:mergeCell ref="B46:L46"/>
-    <x:mergeCell ref="B47:L47"/>
     <x:mergeCell ref="A49:D49"/>
     <x:mergeCell ref="E49:H49"/>
     <x:mergeCell ref="I49:L49"/>
     <x:mergeCell ref="A50:D51"/>
     <x:mergeCell ref="E50:H51"/>
     <x:mergeCell ref="I50:L51"/>
+    <x:mergeCell ref="A43:C43"/>
+    <x:mergeCell ref="D43:L43"/>
+    <x:mergeCell ref="A44:C44"/>
+    <x:mergeCell ref="D44:L44"/>
+    <x:mergeCell ref="A45:C45"/>
+    <x:mergeCell ref="D45:L45"/>
+    <x:mergeCell ref="A46:C46"/>
+    <x:mergeCell ref="D46:L46"/>
+    <x:mergeCell ref="A47:C47"/>
+    <x:mergeCell ref="D47:L47"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="H10:H34">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -1365,7 +1370,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="K5">
-      <x:formula1>"QAR,USD,EUR,GBP,AED,SAR,LKR,INR"</x:formula1>
+      <x:formula1>"USD,EUR,GBP,CAD,AUD,NZD,CHF,JPY,CNY,HKD,SGD,INR,AED,SAR,QAR,LKR,ZAR,BRL,MXN"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B6">
       <x:formula1>"Stock Variance,Damage,Expiry,Write-off,UOM Correction,Location Correction,System Error,Other"</x:formula1>
@@ -1399,81 +1404,126 @@
       <x:c r="E1" s="57"/>
       <x:c r="F1" s="57"/>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="55" customHeight="1">
       <x:c r="A3" s="33" t="str">
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B3" s="26" t="str">
-        <x:v>Use this form after a stock discrepancy or other adjustment requirement has been verified and approved.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="34" customHeight="1">
+        <x:v>Prepare after investigation; obtain approval before posting. The calculated difference is a proposed correction, not authorization.</x:v>
+      </x:c>
+      <x:c r="C3" s="26"/>
+      <x:c r="D3" s="26"/>
+      <x:c r="E3" s="26"/>
+      <x:c r="F3" s="26"/>
+    </x:row>
+    <x:row r="4" ht="55" customHeight="1">
       <x:c r="A4" s="33" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="26" t="str">
         <x:v>Complete the document information including warehouse, date, reference, preparer and adjustment type.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="C4" s="26"/>
+      <x:c r="D4" s="26"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+    </x:row>
+    <x:row r="5" ht="55" customHeight="1">
       <x:c r="A5" s="33" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="26" t="str">
-        <x:v>Enter SKU, description, location, UOM, current system quantity and verified physical quantity.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
+        <x:v>Use the same SKU, location, stock status, UOM and cutoff for both quantities. Enter 0 for a verified zero; leave unknown quantities blank.</x:v>
+      </x:c>
+      <x:c r="C5" s="26"/>
+      <x:c r="D5" s="26"/>
+      <x:c r="E5" s="26"/>
+      <x:c r="F5" s="26"/>
+    </x:row>
+    <x:row r="6" ht="55" customHeight="1">
       <x:c r="A6" s="33" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="26" t="str">
         <x:v>Adjustment Qty is calculated automatically as Verified Qty - System Qty.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="C6" s="26"/>
+      <x:c r="D6" s="26"/>
+      <x:c r="E6" s="26"/>
+      <x:c r="F6" s="26"/>
+    </x:row>
+    <x:row r="7" ht="55" customHeight="1">
       <x:c r="A7" s="33" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>Enter Unit Cost if you want the workbook to calculate the financial adjustment value.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="34" customHeight="1">
+        <x:v>Select one currency (USD default; no exchange conversion). Enter every unit cost for complete value totals. Missing costs show Incomplete; net value can offset shortages against excesses.</x:v>
+      </x:c>
+      <x:c r="C7" s="26"/>
+      <x:c r="D7" s="26"/>
+      <x:c r="E7" s="26"/>
+      <x:c r="F7" s="26"/>
+    </x:row>
+    <x:row r="8" ht="55" customHeight="1">
       <x:c r="A8" s="33" t="str">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
         <x:v>Select a reason code and write a clear explanation for each adjustment line.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="C8" s="26"/>
+      <x:c r="D8" s="26"/>
+      <x:c r="E8" s="26"/>
+      <x:c r="F8" s="26"/>
+    </x:row>
+    <x:row r="9" ht="55" customHeight="1">
       <x:c r="A9" s="33" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="26" t="str">
         <x:v>Summarize the investigation, corrective action and preventive action in the control section.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="26"/>
+      <x:c r="F9" s="26"/>
+    </x:row>
+    <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="33" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B10" s="26" t="str">
         <x:v>Obtain the required review and approval before posting the inventory adjustment in your system.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="C10" s="26"/>
+      <x:c r="D10" s="26"/>
+      <x:c r="E10" s="26"/>
+      <x:c r="F10" s="26"/>
+    </x:row>
+    <x:row r="11" ht="55" customHeight="1">
       <x:c r="A11" s="33" t="str">
         <x:v>Control note</x:v>
       </x:c>
       <x:c r="B11" s="26" t="str">
-        <x:v>Keep supporting evidence such as count sheets, variance reports, GRNs, issue notes, transfer documents or photographs according to your business procedure.</x:v>
-      </x:c>
+        <x:v>Keep count and transaction evidence. Correct missing receipts, transfers or UOM errors through the appropriate transaction where possible; do not also post a duplicate quantity adjustment.</x:v>
+      </x:c>
+      <x:c r="C11" s="26"/>
+      <x:c r="D11" s="26"/>
+      <x:c r="E11" s="26"/>
+      <x:c r="F11" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="B3:F3"/>
+    <x:mergeCell ref="B4:F4"/>
+    <x:mergeCell ref="B5:F5"/>
+    <x:mergeCell ref="B6:F6"/>
+    <x:mergeCell ref="B7:F7"/>
+    <x:mergeCell ref="B8:F8"/>
+    <x:mergeCell ref="B9:F9"/>
+    <x:mergeCell ref="B10:F10"/>
+    <x:mergeCell ref="B11:F11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1490,7 +1540,7 @@
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1594,7 +1644,7 @@
         <x:v>-40</x:v>
       </x:c>
       <x:c r="H4" s="26" t="str">
-        <x:v>DAMAGE</x:v>
+        <x:v>Verified shortage</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>